<commit_message>
Calculated quarterly/annual inflation rate, cumulative chained indices, and produced graphs
</commit_message>
<xml_diff>
--- a/Quarter/Predicted_Quarterly_Jevons_Index_Results.xlsx
+++ b/Quarter/Predicted_Quarterly_Jevons_Index_Results.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Predicted_Prices" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Adjacent Predicted Quarters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Model_Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11673,6 +11674,465 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Samples</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>R2_Score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Features_Selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.9174881104070851</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.001396928987205572</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.8957464416415738</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.01165003882632793</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5908263125679816</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.02595928829554638</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5933947452811486</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.02664194303916071</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>37</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2309290173876728</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>40</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.8172914730233158</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0002256392195441915</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>43</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.8548284482188626</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.004320920619870351</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>47</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.8597342382404278</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.002200568073150742</v>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>61</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.7111227734837067</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0002642017853330548</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>67</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.07520713998920181</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.162285782693552</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>71</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.5337033238215315</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.01547648812940777</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>86</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5739816934408316</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.01024736950624317</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>92</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5713239545348321</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.009505400339516887</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>99</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.445183240026284</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0407420549536488</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>102</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5155364519565655</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0267141460458317</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>117</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.558717089921802</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.008342272188604002</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>121</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.5062422720707349</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.007584276871209199</v>
+      </c>
+      <c r="E18" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>129</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.4984193297363935</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.004064780356087861</v>
+      </c>
+      <c r="E19" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>128</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.4949942646141431</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.009347143852108929</v>
+      </c>
+      <c r="E20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>140</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5223376613774526</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.001761477111971307</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>146</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.5258317880848239</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.003012836416271812</v>
+      </c>
+      <c r="E22" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>133</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5776295687038513</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0002518806511539167</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Added coefficients and regression tables
</commit_message>
<xml_diff>
--- a/Quarter/Predicted_Quarterly_Jevons_Index_Results.xlsx
+++ b/Quarter/Predicted_Quarterly_Jevons_Index_Results.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Predicted_Prices" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Adjacent Predicted Quarters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Model_Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Coefficients" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12133,6 +12134,4804 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F199"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Coefficient</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Abs_Coefficient</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CI_Lower</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CI_Upper</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1857637921839924</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1857637921839924</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.05404861489844906</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.6051360399362462</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.07878901228368154</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2412059664904359</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2118917169094785</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.2118917169094785</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.6854904293046815</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1633701740964541</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.1633701740964541</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2988023614202707</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.1525267150265484</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1525267150265484</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.4053010079563933</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.2138592441832249</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2138592441832249</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.08160950504424112</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4099859170698995</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-0.4630402713758578</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3022503534647858</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2020 Q1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.06180546527326223</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.06180546527326223</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.09957552479540883</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.307476385976792</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.02298599828716866</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.02298599828716866</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.01513054425622818</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.1240920227130506</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.1687328406125843</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.08422242961588518</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.08422242961588518</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.172988997763518</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>-0.09676668247771555</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.09676668247771555</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.1703320824368134</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1423367484868813</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1423367484868813</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.07467465610651912</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.2200717469536283</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.04947436202036568</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.04947436202036568</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-0.1685082783774751</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.09447816620285006</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2020 Q2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.1438369161400357</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.2184277587354788</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-0.004423452068108455</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.06893256506690595</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-0.1245338230223286</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.1478072024168907</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-0.2912846520211864</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.07678417849049077</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1252740496940311</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.1252740496940311</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.03876638344918534</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.2225223740815895</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.08374899147921061</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.08374899147921061</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2627867891413901</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2020 Q3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.3504070146472664</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-0.000563339240136646</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.0881918770645094</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-0.1494917371433486</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.1718954997630205</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.03134733022452624</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.03134733022452624</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-0.3112106984516267</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.1268984781324135</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>0.1612378329672517</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.1612378329672517</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.04582839228071055</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.2815430056858093</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0.06826717379416157</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.06826717379416157</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-0.004316500116916339</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.3265986338767513</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2020 Q4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.1407786605190332</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.2634530430614674</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.413328807255099</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-0.1561045163926366</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2021 Q1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0.9313539350119253</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.9313539350119253</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.3776788367724182</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1.780014567023761</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>-0.5065063873159779</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.5065063873159779</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-0.8928087414486655</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.03103099509919548</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>0.386714190202694</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.386714190202694</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.1572930561222504</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.8496137042594514</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>0.08490554192857765</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.08490554192857765</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-0.03768329063711715</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.3316581481434702</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>0.1812276239475903</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.1812276239475903</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-0.2899924825860552</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.3967753377759476</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>0.2487609851222373</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.2487609851222373</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.05754284963277352</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.411454292388197</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>-0.0241215727953903</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.0241215727953903</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-0.1172605074545273</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.09122244037341271</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>0.2032613889097503</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.2032613889097503</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-0.424848967231639</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.6530377644650071</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2021 Q2</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>0.3271007592024814</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.3271007592024814</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.08966441985290811</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.7091636961415635</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>0.8731639137434921</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.8731639137434921</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.5186151795367143</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1.679936046208772</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>-0.3726572317981829</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.3726572317981829</v>
+      </c>
+      <c r="E57" t="n">
+        <v>-0.8685693239487834</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>0.4020323494055918</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.4020323494055918</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.2217866062918087</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.7343101758851553</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0.07505596178797697</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.07505596178797697</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-0.07745237981565072</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.2505301732030164</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>0.1564444056966052</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.1564444056966052</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-0.2039598222917266</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.3191621076920622</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>0.2240215961305959</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.2240215961305959</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.0833376495784322</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.3931564260284228</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>-0.009884654941270892</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.009884654941270892</v>
+      </c>
+      <c r="E62" t="n">
+        <v>-0.1477975634551355</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.1692870180015783</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>0.1077551566874989</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.1077551566874989</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-0.2911807908297063</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.8107519083939552</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2021 Q3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>0.2925840813350163</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.2925840813350163</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.1139120961035168</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.647766279857638</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1.061755436675657</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1.061755436675657</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.6814032915528443</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1.628916912665801</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>-0.453044403561492</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.453044403561492</v>
+      </c>
+      <c r="E66" t="n">
+        <v>-0.8305902825860138</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-0.08596980998564741</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>0.4696091568301163</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.4696091568301163</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.2887253568658609</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.709913611367163</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>0.04480644816339514</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0.04480644816339514</v>
+      </c>
+      <c r="E68" t="n">
+        <v>-0.08090156900213578</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.2002081355678578</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0.1649951444654681</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0.1649951444654681</v>
+      </c>
+      <c r="E69" t="n">
+        <v>-0.3018513766167408</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.3271495395868967</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0.1940681780404903</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.1940681780404903</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.06824679622848794</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.3438117562603907</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>-0.1422033053352867</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.1915986152183971</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0.3687525099413028</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.3687525099413028</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.7645954211831432</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2021 Q4</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0.1972581347974214</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.1972581347974214</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.4770480744367075</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1.173240475610088</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1.173240475610088</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.8535828167299967</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1.659866342073539</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>-0.4699835963646718</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0.4699835963646718</v>
+      </c>
+      <c r="E75" t="n">
+        <v>-0.6761413248322473</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-0.2586315019436738</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>0.5895378468992868</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0.5895378468992868</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.3826061871410921</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.8398910917474263</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>0.04192033261732816</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0.04192033261732816</v>
+      </c>
+      <c r="E77" t="n">
+        <v>-0.08876356245018424</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.2133579135167748</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>0.1962313288277321</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0.1962313288277321</v>
+      </c>
+      <c r="E78" t="n">
+        <v>-0.1335217484035552</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.3576291338680346</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>0.2209119717289076</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.2209119717289076</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.06797155338302245</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.3766463544974631</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>0.004939555870256844</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0.004939555870256844</v>
+      </c>
+      <c r="E80" t="n">
+        <v>-0.1093515276289318</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.154875969387137</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>0.5989497978870932</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0.5989497978870932</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.235279965267097</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.9098735099668035</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2022 Q1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>-0.02271795021240743</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.02271795021240743</v>
+      </c>
+      <c r="E82" t="n">
+        <v>-0.274870862059135</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.2365942764244163</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.2120818897829044</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.1283514875828773</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.1341641323230749</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.1280029574126614</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>0.05224647126007063</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0.05224647126007063</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.326680189630224</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.2653729899980493</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2022 Q2</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>0.4459213235201416</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0.4459213235201416</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0.3442774379000199</v>
+      </c>
+      <c r="F92" t="n">
+        <v>1.200369587697943</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>-0.4726335402394434</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.2026963900958794</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>0.2859652961240194</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0.2859652961240194</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0.1944050473152886</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.6262432147853669</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>0.03864342539579125</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0.03864342539579125</v>
+      </c>
+      <c r="E95" t="n">
+        <v>-0.09643990497538048</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0.1709679820707169</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>0.07252179614283619</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0.07252179614283619</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.2226595653800066</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>0.1223462750763021</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0.1223462750763021</v>
+      </c>
+      <c r="E97" t="n">
+        <v>-0.01488770795102563</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.2604941069093785</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>0.09917168453969603</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0.09917168453969603</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.2322965283963086</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>0.1006195829763146</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0.1006195829763146</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.8026530171164201</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2022 Q3</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>-0.1023420094640609</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0.1023420094640609</v>
+      </c>
+      <c r="E100" t="n">
+        <v>-0.5512253138982136</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>0.564352529881233</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0.564352529881233</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0.4635158927426167</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0.8493393228382478</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>0.002825496298822778</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0.002825496298822778</v>
+      </c>
+      <c r="E102" t="n">
+        <v>-0.2081986409801691</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.1992674643219199</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>0.3903766300319195</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0.3903766300319195</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0.2702414311957289</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.6278903517988969</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>0.06271229684860463</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.06271229684860463</v>
+      </c>
+      <c r="E104" t="n">
+        <v>-0.003472989367675925</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0.201557664172955</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>-0.1652097506452191</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.0977534153442607</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>-0.01913843679932817</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0.01913843679932817</v>
+      </c>
+      <c r="E106" t="n">
+        <v>-0.163568410571306</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0.0519906860820173</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>0.1183350592563079</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0.1183350592563079</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0.01652579511251265</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0.2526112790590811</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>0.1501826385890482</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0.1501826385890482</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0.458636944667219</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2022 Q4</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>-0.2506500740126339</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0.1140748452272229</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>0.4903216617426285</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0.4903216617426285</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0.4429802764297243</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0.748384039607299</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>0.1470359399785711</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0.1470359399785711</v>
+      </c>
+      <c r="E111" t="n">
+        <v>-0.03353888960176347</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0.2581042011054249</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>0.393050063891912</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0.393050063891912</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0.267138675904181</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.5844886298700254</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>0.1344294739626193</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0.1344294739626193</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0.2829080461040188</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>0.004236863994576556</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0.004236863994576556</v>
+      </c>
+      <c r="E114" t="n">
+        <v>-0.1384461812422755</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0.1534555696077269</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>-0.07407887410279967</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0.07407887410279967</v>
+      </c>
+      <c r="E115" t="n">
+        <v>-0.1906224114387359</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.0190783444800419</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>0.07108631469976219</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0.07108631469976219</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0.1858726384968583</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>0.01946393321774164</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0.01946393321774164</v>
+      </c>
+      <c r="E117" t="n">
+        <v>-0.1016008545144935</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.2792654008018065</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>0.003227027472922985</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0.003227027472922985</v>
+      </c>
+      <c r="E118" t="n">
+        <v>-0.183413431880412</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.228305787645327</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>0.2896066090963929</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0.2896066090963929</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.3406438088076964</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.6184341079620058</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>0.0956462226868032</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0.0956462226868032</v>
+      </c>
+      <c r="E120" t="n">
+        <v>-0.08043932989650557</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.2018784321954755</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>0.2652701404145971</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0.2652701404145971</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0.2053490466512259</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.5115184168450986</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>0.0608990408400144</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.0608990408400144</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.2527895982222923</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.1687160693732263</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" t="n">
+        <v>-0.1511608505532172</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.02288123935494765</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" t="n">
+        <v>-0.05824209086926082</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.1236693228787035</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.2198262247005623</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.1832126536772278</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>0.3556184397121477</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.3556184397121477</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.35360128497254</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.6214462003534453</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>0.09138265144668266</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.09138265144668266</v>
+      </c>
+      <c r="E129" t="n">
+        <v>-0.04404017573666069</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.2066487893252846</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>0.3298975915067728</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.3298975915067728</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.2518728306196721</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0.5307195116590659</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>0.07737479331339145</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.07737479331339145</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.2345969446301637</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.1709938227504996</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>-0.1241742217464924</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0.04631767544872546</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>-0.08630675165125624</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0.09188968112546554</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>-0.1492749234113633</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0.1208483065150474</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0.2205369165793573</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>0.4723346202479389</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.4723346202479389</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.4155290796996186</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0.6463067660760099</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>0.07014772446520236</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0.07014772446520236</v>
+      </c>
+      <c r="E138" t="n">
+        <v>-0.01741999242853782</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0.1768631894497099</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>0.3742123077884833</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0.3742123077884833</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.2607772135953893</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.5231144937249713</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>0.1402514436929242</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0.1402514436929242</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.02821622746859481</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0.2611396932540289</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>0.05096134340047236</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0.05096134340047236</v>
+      </c>
+      <c r="E141" t="n">
+        <v>-0.06485764384790894</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0.1730192377867401</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>-0.06803794601474282</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0.06803794601474282</v>
+      </c>
+      <c r="E142" t="n">
+        <v>-0.1566165525738658</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>0.004693271727592019</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0.004693271727592019</v>
+      </c>
+      <c r="E143" t="n">
+        <v>-0.09019199140471906</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.1202542412603088</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>-0.1215842067613413</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0.1740680203161866</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>0.0200890683108282</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.0200890683108282</v>
+      </c>
+      <c r="E145" t="n">
+        <v>-0.1156330328144344</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0.1824502517397567</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>0.4309569405308885</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.4309569405308885</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.3533862808490795</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0.5982983410106342</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0.06306617086596651</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0.06306617086596651</v>
+      </c>
+      <c r="E147" t="n">
+        <v>-0.09330422276661755</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0.1903503163710812</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0.3949672565606416</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0.3949672565606416</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0.272556381792994</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0.5555612757370376</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>0.1062874579292347</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.1062874579292347</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0.241021340478615</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>0.03324572015388162</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.03324572015388162</v>
+      </c>
+      <c r="E150" t="n">
+        <v>-0.08657770368336738</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0.146623037103302</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>-0.08318593442535961</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.08318593442535961</v>
+      </c>
+      <c r="E151" t="n">
+        <v>-0.1782565695202081</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>-0.01435825775771297</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0.01435825775771297</v>
+      </c>
+      <c r="E152" t="n">
+        <v>-0.1102643238465887</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0.07844506114666752</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>0.0334011008799985</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0.0334011008799985</v>
+      </c>
+      <c r="E153" t="n">
+        <v>-0.09080421428823864</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0.2324562658953494</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>-0.1497872535156528</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0.151305631787712</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>0.4563494406479617</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0.4563494406479617</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0.3627587388282498</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0.6406934751311274</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>0.04603229928929434</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0.04603229928929434</v>
+      </c>
+      <c r="E156" t="n">
+        <v>-0.1423388026147983</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.1598582597857418</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>0.369912540941521</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0.369912540941521</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0.2191710244498077</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0.5279500044200076</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>0.1593856520033927</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0.1593856520033927</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0.04936701515933652</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0.2973575503848574</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>0.07015798996763922</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0.07015798996763922</v>
+      </c>
+      <c r="E159" t="n">
+        <v>-0.04383894240157622</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0.1890964491001826</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>-0.06376498791720282</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0.06376498791720282</v>
+      </c>
+      <c r="E160" t="n">
+        <v>-0.1421714268893625</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0.01489661778911441</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>-0.02060515616784358</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0.02060515616784358</v>
+      </c>
+      <c r="E161" t="n">
+        <v>-0.1308520146810297</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0.06475082476677954</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>0.05117475819083966</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0.05117475819083966</v>
+      </c>
+      <c r="E162" t="n">
+        <v>-0.07593410285650237</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0.2474745490974148</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>0.02246650301515702</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0.02246650301515702</v>
+      </c>
+      <c r="E163" t="n">
+        <v>-0.1250032459470009</v>
+      </c>
+      <c r="F163" t="n">
+        <v>0.1935163875170093</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>0.4255442114006846</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0.4255442114006846</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0.3578996497478709</v>
+      </c>
+      <c r="F164" t="n">
+        <v>0.5998480616817814</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>0.05499853967960792</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0.05499853967960792</v>
+      </c>
+      <c r="E165" t="n">
+        <v>-0.09185424010822463</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0.1644755706441698</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>0.3573859912577329</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0.3573859912577329</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0.2247834713646746</v>
+      </c>
+      <c r="F166" t="n">
+        <v>0.5266429571143394</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>0.1459601812445006</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0.1459601812445006</v>
+      </c>
+      <c r="E167" t="n">
+        <v>0.03189127050060286</v>
+      </c>
+      <c r="F167" t="n">
+        <v>0.2875454499112672</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>0.05663529226961636</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0.05663529226961636</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" t="n">
+        <v>0.1657338001974212</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>-0.03728585269017264</v>
+      </c>
+      <c r="D169" t="n">
+        <v>0.03728585269017264</v>
+      </c>
+      <c r="E169" t="n">
+        <v>-0.1260878528876527</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0.01849044624342408</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>-0.005708688530711384</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0.005708688530711384</v>
+      </c>
+      <c r="E170" t="n">
+        <v>-0.121843378295389</v>
+      </c>
+      <c r="F170" t="n">
+        <v>0.07125464566866092</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0.02358547792542121</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0.02358547792542121</v>
+      </c>
+      <c r="E171" t="n">
+        <v>-0.1126890051879821</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0.2164992448872527</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>0.01390750367657731</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0.01390750367657731</v>
+      </c>
+      <c r="E172" t="n">
+        <v>-0.108320266916728</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0.1616418783093524</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>0.4827416901240673</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0.4827416901240673</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0.3730821281028855</v>
+      </c>
+      <c r="F173" t="n">
+        <v>0.6366304122434899</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>0.04444024064023925</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0.04444024064023925</v>
+      </c>
+      <c r="E174" t="n">
+        <v>-0.1404327369880334</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0.1693284564920854</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>0.3836245611943112</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0.3836245611943112</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0.2450670672061087</v>
+      </c>
+      <c r="F175" t="n">
+        <v>0.5357752464737158</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>0.1422635959888507</v>
+      </c>
+      <c r="D176" t="n">
+        <v>0.1422635959888507</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0.02251942943056369</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0.2735292070771808</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>0.04825088588234584</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0.04825088588234584</v>
+      </c>
+      <c r="E177" t="n">
+        <v>-0.0546376906688896</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0.170315477396603</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>-0.09315118261139367</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0.09315118261139367</v>
+      </c>
+      <c r="E178" t="n">
+        <v>-0.1692296721212916</v>
+      </c>
+      <c r="F178" t="n">
+        <v>-0.002916650038349188</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>-0.05181330519401679</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0.05181330519401679</v>
+      </c>
+      <c r="E179" t="n">
+        <v>-0.1563921647449814</v>
+      </c>
+      <c r="F179" t="n">
+        <v>0.04141349710474277</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>0.08714349704811487</v>
+      </c>
+      <c r="D180" t="n">
+        <v>0.08714349704811487</v>
+      </c>
+      <c r="E180" t="n">
+        <v>-0.04414278910867144</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0.2732042197852474</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>0</v>
+      </c>
+      <c r="D181" t="n">
+        <v>0</v>
+      </c>
+      <c r="E181" t="n">
+        <v>-0.1474788147220487</v>
+      </c>
+      <c r="F181" t="n">
+        <v>0.1696184117918043</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>0.4525039609227554</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.4525039609227554</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0.3436282026775461</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0.6334622807865218</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>0</v>
+      </c>
+      <c r="D183" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" t="n">
+        <v>-0.1746831366770479</v>
+      </c>
+      <c r="F183" t="n">
+        <v>0.1260602305328002</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>0.3861329390385662</v>
+      </c>
+      <c r="D184" t="n">
+        <v>0.3861329390385662</v>
+      </c>
+      <c r="E184" t="n">
+        <v>0.2610106016174176</v>
+      </c>
+      <c r="F184" t="n">
+        <v>0.5243075956815083</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>0.1335916354003166</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0.1335916354003166</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0.01704848494128492</v>
+      </c>
+      <c r="F185" t="n">
+        <v>0.267283271789012</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>0.06240712962375154</v>
+      </c>
+      <c r="D186" t="n">
+        <v>0.06240712962375154</v>
+      </c>
+      <c r="E186" t="n">
+        <v>-0.02904514060490312</v>
+      </c>
+      <c r="F186" t="n">
+        <v>0.1876114045471927</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>-0.06179798873279796</v>
+      </c>
+      <c r="D187" t="n">
+        <v>0.06179798873279796</v>
+      </c>
+      <c r="E187" t="n">
+        <v>-0.1454793911583435</v>
+      </c>
+      <c r="F187" t="n">
+        <v>0.02755679996817816</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>-0.04598068204367296</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0.04598068204367296</v>
+      </c>
+      <c r="E188" t="n">
+        <v>-0.1496080902406929</v>
+      </c>
+      <c r="F188" t="n">
+        <v>0.02558497704783524</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>0.1115271842537083</v>
+      </c>
+      <c r="D189" t="n">
+        <v>0.1115271842537083</v>
+      </c>
+      <c r="E189" t="n">
+        <v>-0.04164236773080721</v>
+      </c>
+      <c r="F189" t="n">
+        <v>0.2752099917412126</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>0.0309966125833228</v>
+      </c>
+      <c r="D190" t="n">
+        <v>0.0309966125833228</v>
+      </c>
+      <c r="E190" t="n">
+        <v>-0.1170631570753333</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0.2305123218268696</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>is_ios</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>0.5250038078739722</v>
+      </c>
+      <c r="D191" t="n">
+        <v>0.5250038078739722</v>
+      </c>
+      <c r="E191" t="n">
+        <v>0.3985165045240442</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0.6636813142362759</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>mobile_weight_numeric</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>-0.0949482932907858</v>
+      </c>
+      <c r="D192" t="n">
+        <v>0.0949482932907858</v>
+      </c>
+      <c r="E192" t="n">
+        <v>-0.2850336668605579</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0.01712282726101078</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>ram_mem_numeric</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>0.3934167481601822</v>
+      </c>
+      <c r="D193" t="n">
+        <v>0.3934167481601822</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0.1999043633950023</v>
+      </c>
+      <c r="F193" t="n">
+        <v>0.5549057215074817</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>front_camera_mp</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>0.132389551382991</v>
+      </c>
+      <c r="D194" t="n">
+        <v>0.132389551382991</v>
+      </c>
+      <c r="E194" t="n">
+        <v>-0.02349092437895339</v>
+      </c>
+      <c r="F194" t="n">
+        <v>0.2596480302674271</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>max_mp_numeric</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>0.07101891839331902</v>
+      </c>
+      <c r="D195" t="n">
+        <v>0.07101891839331902</v>
+      </c>
+      <c r="E195" t="n">
+        <v>-0.06070652591979152</v>
+      </c>
+      <c r="F195" t="n">
+        <v>0.208121443352837</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>num_cameras_numeric</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>-0.05538260764949894</v>
+      </c>
+      <c r="D196" t="n">
+        <v>0.05538260764949894</v>
+      </c>
+      <c r="E196" t="n">
+        <v>-0.1229589610615807</v>
+      </c>
+      <c r="F196" t="n">
+        <v>0.03632703097905425</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>processor_level_encoded</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>-0.06976673360940663</v>
+      </c>
+      <c r="D197" t="n">
+        <v>0.06976673360940663</v>
+      </c>
+      <c r="E197" t="n">
+        <v>-0.1433191726592311</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0.02797653336268166</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>battery_capacity_numeric</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>0.1286170105398614</v>
+      </c>
+      <c r="D198" t="n">
+        <v>0.1286170105398614</v>
+      </c>
+      <c r="E198" t="n">
+        <v>-0.02416983176987936</v>
+      </c>
+      <c r="F198" t="n">
+        <v>0.338221438373267</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>screen_size_numeric</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>0.1703793500171292</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0.1703793500171292</v>
+      </c>
+      <c r="E199" t="n">
+        <v>0.01113736041798686</v>
+      </c>
+      <c r="F199" t="n">
+        <v>0.3343540567429609</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>